<commit_message>
fix: excels import based on different sheet names and new ones
</commit_message>
<xml_diff>
--- a/public/files/IQMY-Alpro Code Mapping Document 07Aug2025-ver2.0-NS.xlsx
+++ b/public/files/IQMY-Alpro Code Mapping Document 07Aug2025-ver2.0-NS.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pathologyasia-my.sharepoint.com/personal/iqmy0959_pathologyasia_com/Documents/PROJECT - Integration/Alpro/Mapping/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\blood-stream-v1\public\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1630" documentId="8_{979185E3-AEED-4204-9A49-BEB87E4494B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A5EE702-D6A2-4CE8-9F8D-C001DAE9D2B9}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{092FE06D-D5EC-4179-827D-C9136176BAF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{90924F02-D7F6-4704-901E-FE125CE86CD4}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{90924F02-D7F6-4704-901E-FE125CE86CD4}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Panel Code" sheetId="11" r:id="rId1"/>
     <sheet name="2. Profile Code" sheetId="3" r:id="rId2"/>
     <sheet name="3. Doctor Code" sheetId="4" r:id="rId3"/>
-    <sheet name="4. Tag On (TON)" sheetId="5" r:id="rId4"/>
-    <sheet name="5. Tag On (QON)" sheetId="10" r:id="rId5"/>
+    <sheet name="4. Tag On" sheetId="5" r:id="rId4"/>
+    <sheet name="5. Tag On" sheetId="10" r:id="rId5"/>
     <sheet name="6. Reported Test" sheetId="6" r:id="rId6"/>
     <sheet name="7. Bill Code" sheetId="8" r:id="rId7"/>
     <sheet name="8. Department Code" sheetId="12" r:id="rId8"/>
@@ -37,8 +37,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -46,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9065" uniqueCount="1878">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9065" uniqueCount="1879">
   <si>
     <t>PANEL</t>
   </si>
@@ -5384,21 +5382,12 @@
     <t>FT2</t>
   </si>
   <si>
-    <t>Department</t>
-  </si>
-  <si>
     <t>PSA (GE)</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>TON Name</t>
-  </si>
-  <si>
-    <t>CODE</t>
-  </si>
-  <si>
     <t>QFX</t>
   </si>
   <si>
@@ -5507,9 +5496,6 @@
     <t>HISTOLOGY</t>
   </si>
   <si>
-    <t>QON Name</t>
-  </si>
-  <si>
     <t>EN</t>
   </si>
   <si>
@@ -5688,6 +5674,21 @@
   </si>
   <si>
     <t>LIS Value</t>
+  </si>
+  <si>
+    <t>PANEL CODE</t>
+  </si>
+  <si>
+    <t>PANEL NAME</t>
+  </si>
+  <si>
+    <t>DEPARTMENT</t>
+  </si>
+  <si>
+    <t>TAG ON CODE</t>
+  </si>
+  <si>
+    <t>TAG ON NAME</t>
   </si>
 </sst>
 </file>
@@ -6026,7 +6027,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -6132,7 +6133,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -6142,106 +6142,11 @@
   <dxfs count="30">
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF156082"/>
-          <bgColor rgb="FF156082"/>
         </patternFill>
       </fill>
     </dxf>
@@ -6334,6 +6239,30 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF156082"/>
+          <bgColor rgb="FF156082"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -6646,6 +6575,77 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -6660,40 +6660,40 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{6F3870D0-158B-4679-A5F5-F1DBFEB21CF1}" name="Table8" displayName="Table8" ref="A1:C87" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{6F3870D0-158B-4679-A5F5-F1DBFEB21CF1}" name="Table8" displayName="Table8" ref="A1:C87" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
   <autoFilter ref="A1:C87" xr:uid="{6F3870D0-158B-4679-A5F5-F1DBFEB21CF1}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B86">
     <sortCondition ref="A1:A86"/>
   </sortState>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{65309BB8-FC15-45B0-8344-F8AB1E4256ED}" name="PANEL" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{04FEB7BD-102A-42ED-B2E8-C1C8B49B6170}" name="NAME" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{AC55274A-1F36-4E8B-B333-3C871B1CE840}" name="Department" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{65309BB8-FC15-45B0-8344-F8AB1E4256ED}" name="PANEL CODE" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{04FEB7BD-102A-42ED-B2E8-C1C8B49B6170}" name="PANEL NAME" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{AC55274A-1F36-4E8B-B333-3C871B1CE840}" name="DEPARTMENT" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1FA2374D-F190-4369-B6B2-F43C4D28D00E}" name="Table4" displayName="Table4" ref="A1:F251" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1FA2374D-F190-4369-B6B2-F43C4D28D00E}" name="Table4" displayName="Table4" ref="A1:F251" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
   <autoFilter ref="A1:F251" xr:uid="{1FA2374D-F190-4369-B6B2-F43C4D28D00E}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F250">
     <sortCondition ref="A1:A250"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{A00151FA-7997-4B12-AD72-EE06E507D1A0}" name="LIS Profile/Package Code " dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{D6281925-FD6E-4643-B9C7-DEE95733C11C}" name="LIS Profile  Test Name " dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{AA189E91-AB2A-4705-AE32-9EFD22927DD1}" name="Panel " dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{B0BD8119-6312-406E-98FD-86E4C2BA1E04}" name="Panel Name" dataDxfId="24"/>
-    <tableColumn id="6" xr3:uid="{7B795EC0-4B03-46DF-888D-5081E21C0FB2}" name="Lab Category" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{67A540FC-1789-479A-9ADE-8E9431B01722}" name="Remarks" dataDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{A00151FA-7997-4B12-AD72-EE06E507D1A0}" name="LIS Profile/Package Code " dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{D6281925-FD6E-4643-B9C7-DEE95733C11C}" name="LIS Profile  Test Name " dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{AA189E91-AB2A-4705-AE32-9EFD22927DD1}" name="Panel " dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{B0BD8119-6312-406E-98FD-86E4C2BA1E04}" name="Panel Name" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{7B795EC0-4B03-46DF-888D-5081E21C0FB2}" name="Lab Category" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{67A540FC-1789-479A-9ADE-8E9431B01722}" name="Remarks" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4EE06AA4-F75E-428B-BE09-32159E280165}" name="Table1" displayName="Table1" ref="A1:E235" totalsRowShown="0" headerRowDxfId="21" dataDxfId="19" headerRowBorderDxfId="20" tableBorderDxfId="18" totalsRowBorderDxfId="17" headerRowCellStyle="Normal 2" dataCellStyle="Normal 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4EE06AA4-F75E-428B-BE09-32159E280165}" name="Table1" displayName="Table1" ref="A1:E235" totalsRowShown="0" headerRowDxfId="16" dataDxfId="14" headerRowBorderDxfId="15" tableBorderDxfId="13" totalsRowBorderDxfId="12" headerRowCellStyle="Normal 2" dataCellStyle="Normal 2">
   <autoFilter ref="A1:E235" xr:uid="{4EE06AA4-F75E-428B-BE09-32159E280165}">
     <filterColumn colId="1">
       <filters>
@@ -6702,11 +6702,11 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="8" xr3:uid="{6897669A-DECC-418C-BC45-051847085CFB}" name="CLINIC/PHARMACY" dataDxfId="16" dataCellStyle="Normal 2"/>
-    <tableColumn id="1" xr3:uid="{3FD8DE49-91B1-4466-83B5-511E172BA616}" name="Dr Code" dataDxfId="15" dataCellStyle="Normal 2"/>
-    <tableColumn id="4" xr3:uid="{FF5F237B-ED13-4A20-8D5A-303F9A6CDA74}" name="Doctor Name" dataDxfId="14" dataCellStyle="Normal 2"/>
-    <tableColumn id="5" xr3:uid="{50C700EE-6AD3-42B8-A01E-BF643BBECD0C}" name="Outlet" dataDxfId="13" dataCellStyle="Normal 2"/>
-    <tableColumn id="6" xr3:uid="{AE623DDB-C521-44E3-8F9A-1BCC232B7174}" name="Address" dataDxfId="12" dataCellStyle="Normal 2"/>
+    <tableColumn id="8" xr3:uid="{6897669A-DECC-418C-BC45-051847085CFB}" name="CLINIC/PHARMACY" dataDxfId="11" dataCellStyle="Normal 2"/>
+    <tableColumn id="1" xr3:uid="{3FD8DE49-91B1-4466-83B5-511E172BA616}" name="Dr Code" dataDxfId="10" dataCellStyle="Normal 2"/>
+    <tableColumn id="4" xr3:uid="{FF5F237B-ED13-4A20-8D5A-303F9A6CDA74}" name="Doctor Name" dataDxfId="9" dataCellStyle="Normal 2"/>
+    <tableColumn id="5" xr3:uid="{50C700EE-6AD3-42B8-A01E-BF643BBECD0C}" name="Outlet" dataDxfId="8" dataCellStyle="Normal 2"/>
+    <tableColumn id="6" xr3:uid="{AE623DDB-C521-44E3-8F9A-1BCC232B7174}" name="Address" dataDxfId="7" dataCellStyle="Normal 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6719,10 +6719,10 @@
     <sortCondition ref="C1:C56"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{2A8BE10E-239D-4467-A7A0-4B3FD217DE4A}" name="CODE"/>
-    <tableColumn id="2" xr3:uid="{30840D67-A499-42FE-9598-F48A512F0ED0}" name="NAME"/>
-    <tableColumn id="3" xr3:uid="{8C5E1C69-8405-4413-B972-593768BF95AD}" name="TON"/>
-    <tableColumn id="4" xr3:uid="{466271C4-4E15-4689-830C-0678054E2E40}" name="TON Name"/>
+    <tableColumn id="1" xr3:uid="{2A8BE10E-239D-4467-A7A0-4B3FD217DE4A}" name="PANEL CODE"/>
+    <tableColumn id="2" xr3:uid="{30840D67-A499-42FE-9598-F48A512F0ED0}" name="PANEL NAME"/>
+    <tableColumn id="3" xr3:uid="{8C5E1C69-8405-4413-B972-593768BF95AD}" name="TAG ON CODE"/>
+    <tableColumn id="4" xr3:uid="{466271C4-4E15-4689-830C-0678054E2E40}" name="TAG ON NAME"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6732,23 +6732,23 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DDED538B-5899-4C52-AB52-5094272A1985}" name="Table16" displayName="Table16" ref="A1:D60" totalsRowShown="0">
   <autoFilter ref="A1:D60" xr:uid="{DDED538B-5899-4C52-AB52-5094272A1985}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{D25F724A-DACE-4F63-88EC-2B84DA7FD993}" name="CODE"/>
-    <tableColumn id="2" xr3:uid="{C9D9E5F5-C3CF-477E-886D-609B7658329A}" name="NAME"/>
-    <tableColumn id="3" xr3:uid="{778EBA27-D32A-49A9-A1E2-D30D9ED05307}" name="QON"/>
-    <tableColumn id="4" xr3:uid="{7E4CB048-159B-4494-B211-FD3EBB518C4F}" name="QON Name"/>
+    <tableColumn id="1" xr3:uid="{D25F724A-DACE-4F63-88EC-2B84DA7FD993}" name="PANEL CODE"/>
+    <tableColumn id="2" xr3:uid="{C9D9E5F5-C3CF-477E-886D-609B7658329A}" name="PANEL NAME"/>
+    <tableColumn id="3" xr3:uid="{778EBA27-D32A-49A9-A1E2-D30D9ED05307}" name="TAG ON CODE"/>
+    <tableColumn id="4" xr3:uid="{7E4CB048-159B-4494-B211-FD3EBB518C4F}" name="TAG ON NAME"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{81037DEF-91E8-4677-A7D0-8E7233D94459}" name="Table10" displayName="Table10" ref="A1:D29" totalsRowShown="0" headerRowDxfId="6" dataDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{81037DEF-91E8-4677-A7D0-8E7233D94459}" name="Table10" displayName="Table10" ref="A1:D29" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
   <autoFilter ref="A1:D29" xr:uid="{81037DEF-91E8-4677-A7D0-8E7233D94459}"/>
   <tableColumns count="4">
-    <tableColumn id="4" xr3:uid="{F9917280-ABD9-429E-9C83-CB7E5D95D82E}" name="External Value IN" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{003D68F2-344B-4792-9DA0-365F3FB81707}" name="Externa Value Out" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{C4D72C0A-5D3C-4A75-BA1D-5E8E8C6CA657}" name="LIS Value" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{A2A6A625-5D58-4D3C-B19D-D30939D0CFCE}" name="Description" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{F9917280-ABD9-429E-9C83-CB7E5D95D82E}" name="External Value IN" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{003D68F2-344B-4792-9DA0-365F3FB81707}" name="Externa Value Out" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{C4D72C0A-5D3C-4A75-BA1D-5E8E8C6CA657}" name="LIS Value" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{A2A6A625-5D58-4D3C-B19D-D30939D0CFCE}" name="Description" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -7043,7 +7043,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -7052,22 +7052,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FB29017-77A3-4886-80D9-E9B595B5878B}">
   <dimension ref="A1:C257"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="8.36328125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="29.6328125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="23.81640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.33203125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="29.6640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="23.77734375" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="44" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="44" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="44" t="s">
-        <v>1776</v>
+      <c r="A1" s="43" t="s">
+        <v>1874</v>
+      </c>
+      <c r="B1" s="43" t="s">
+        <v>1875</v>
+      </c>
+      <c r="C1" s="43" t="s">
+        <v>1876</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -7642,7 +7642,7 @@
         <v>1732</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="20.5" customHeight="1">
+    <row r="54" spans="1:3" ht="20.55" customHeight="1">
       <c r="A54" s="2" t="s">
         <v>77</v>
       </c>
@@ -8012,15 +8012,15 @@
       <c r="B87" s="2" t="s">
         <v>1113</v>
       </c>
-      <c r="C87" s="43" t="s">
+      <c r="C87" s="2" t="s">
         <v>1743</v>
       </c>
     </row>
-    <row r="93" spans="1:3" ht="18.5" customHeight="1"/>
-    <row r="257" ht="11.5" customHeight="1"/>
+    <row r="93" spans="1:3" ht="18.45" customHeight="1"/>
+    <row r="257" ht="11.55" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="5" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -8032,16 +8032,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F4ED829-E96E-4333-996E-27CFBED2FDE1}">
   <dimension ref="A1:H251"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="23.81640625" customWidth="1"/>
-    <col min="2" max="2" width="21.26953125" customWidth="1"/>
-    <col min="3" max="3" width="7.90625" customWidth="1"/>
-    <col min="4" max="4" width="26.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.81640625" style="34" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.77734375" customWidth="1"/>
+    <col min="2" max="2" width="21.21875" customWidth="1"/>
+    <col min="3" max="3" width="7.88671875" customWidth="1"/>
+    <col min="4" max="4" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.77734375" style="34" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="37" customHeight="1">
+    <row r="1" spans="1:6" ht="37.049999999999997" customHeight="1">
       <c r="A1" s="32" t="s">
         <v>156</v>
       </c>
@@ -10611,7 +10611,7 @@
         <v>1739</v>
       </c>
     </row>
-    <row r="152" spans="1:5" ht="1" customHeight="1">
+    <row r="152" spans="1:5" ht="1.05" customHeight="1">
       <c r="A152" t="s">
         <v>52</v>
       </c>
@@ -12299,7 +12299,7 @@
         <v>129</v>
       </c>
       <c r="B251" s="37" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
       <c r="C251" s="37" t="s">
         <v>129</v>
@@ -12313,7 +12313,7 @@
       <c r="F251" s="37"/>
       <c r="G251" s="37"/>
       <c r="H251" s="38" t="s">
-        <v>1778</v>
+        <v>1777</v>
       </c>
     </row>
   </sheetData>
@@ -12328,14 +12328,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01D8B73B-281E-49E1-9ED7-16F79163D9A8}">
   <dimension ref="A1:E235"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="18.6328125" style="6" customWidth="1"/>
-    <col min="2" max="2" width="8.7265625" style="11"/>
-    <col min="3" max="3" width="21.36328125" style="11" customWidth="1"/>
-    <col min="4" max="4" width="32.81640625" style="14" customWidth="1"/>
-    <col min="5" max="5" width="48.54296875" style="12" customWidth="1"/>
-    <col min="6" max="16384" width="8.7265625" style="7"/>
+    <col min="1" max="1" width="18.6640625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="8.77734375" style="11"/>
+    <col min="3" max="3" width="21.33203125" style="11" customWidth="1"/>
+    <col min="4" max="4" width="32.77734375" style="14" customWidth="1"/>
+    <col min="5" max="5" width="48.5546875" style="12" customWidth="1"/>
+    <col min="6" max="16384" width="8.77734375" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -12355,7 +12355,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="29" hidden="1">
+    <row r="2" spans="1:5" ht="28.8" hidden="1">
       <c r="A2" s="19" t="s">
         <v>407</v>
       </c>
@@ -12372,7 +12372,7 @@
         <v>1274</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="29" hidden="1">
+    <row r="3" spans="1:5" ht="28.8" hidden="1">
       <c r="A3" s="19" t="s">
         <v>407</v>
       </c>
@@ -12389,7 +12389,7 @@
         <v>1276</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="29" hidden="1">
+    <row r="4" spans="1:5" ht="28.8" hidden="1">
       <c r="A4" s="19" t="s">
         <v>407</v>
       </c>
@@ -12406,7 +12406,7 @@
         <v>1278</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="29" hidden="1">
+    <row r="5" spans="1:5" ht="28.8" hidden="1">
       <c r="A5" s="19" t="s">
         <v>407</v>
       </c>
@@ -12423,7 +12423,7 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="29" hidden="1">
+    <row r="6" spans="1:5" ht="28.8" hidden="1">
       <c r="A6" s="19" t="s">
         <v>407</v>
       </c>
@@ -12457,7 +12457,7 @@
         <v>1284</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="29" hidden="1">
+    <row r="8" spans="1:5" hidden="1">
       <c r="A8" s="19" t="s">
         <v>407</v>
       </c>
@@ -12474,7 +12474,7 @@
         <v>1286</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="29" hidden="1">
+    <row r="9" spans="1:5" ht="28.8" hidden="1">
       <c r="A9" s="19" t="s">
         <v>407</v>
       </c>
@@ -12491,7 +12491,7 @@
         <v>1288</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="29" hidden="1">
+    <row r="10" spans="1:5" ht="28.8" hidden="1">
       <c r="A10" s="19" t="s">
         <v>407</v>
       </c>
@@ -12508,7 +12508,7 @@
         <v>1290</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="29" hidden="1">
+    <row r="11" spans="1:5" ht="28.8" hidden="1">
       <c r="A11" s="19" t="s">
         <v>407</v>
       </c>
@@ -12525,7 +12525,7 @@
         <v>1292</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="29" hidden="1">
+    <row r="12" spans="1:5" ht="28.8" hidden="1">
       <c r="A12" s="19" t="s">
         <v>407</v>
       </c>
@@ -12542,7 +12542,7 @@
         <v>1294</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="29" hidden="1">
+    <row r="13" spans="1:5" ht="28.8" hidden="1">
       <c r="A13" s="19" t="s">
         <v>407</v>
       </c>
@@ -12559,7 +12559,7 @@
         <v>1296</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="29" hidden="1">
+    <row r="14" spans="1:5" ht="28.8" hidden="1">
       <c r="A14" s="19" t="s">
         <v>407</v>
       </c>
@@ -12576,7 +12576,7 @@
         <v>1298</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="29" hidden="1">
+    <row r="15" spans="1:5" ht="28.8" hidden="1">
       <c r="A15" s="19" t="s">
         <v>407</v>
       </c>
@@ -12593,7 +12593,7 @@
         <v>1300</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="29" hidden="1">
+    <row r="16" spans="1:5" ht="28.8" hidden="1">
       <c r="A16" s="19" t="s">
         <v>407</v>
       </c>
@@ -12610,7 +12610,7 @@
         <v>1302</v>
       </c>
     </row>
-    <row r="17" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="17" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A17" s="19" t="s">
         <v>407</v>
       </c>
@@ -12627,7 +12627,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="18" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="18" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A18" s="19" t="s">
         <v>407</v>
       </c>
@@ -12644,7 +12644,7 @@
         <v>1306</v>
       </c>
     </row>
-    <row r="19" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="19" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A19" s="19" t="s">
         <v>407</v>
       </c>
@@ -12661,7 +12661,7 @@
         <v>1308</v>
       </c>
     </row>
-    <row r="20" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="20" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A20" s="19" t="s">
         <v>407</v>
       </c>
@@ -12695,7 +12695,7 @@
         <v>1312</v>
       </c>
     </row>
-    <row r="22" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="22" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A22" s="19" t="s">
         <v>407</v>
       </c>
@@ -12712,7 +12712,7 @@
         <v>1314</v>
       </c>
     </row>
-    <row r="23" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="23" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A23" s="19" t="s">
         <v>407</v>
       </c>
@@ -12729,7 +12729,7 @@
         <v>1316</v>
       </c>
     </row>
-    <row r="24" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="24" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A24" s="19" t="s">
         <v>407</v>
       </c>
@@ -12746,7 +12746,7 @@
         <v>1318</v>
       </c>
     </row>
-    <row r="25" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="25" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A25" s="19" t="s">
         <v>407</v>
       </c>
@@ -12763,7 +12763,7 @@
         <v>1320</v>
       </c>
     </row>
-    <row r="26" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="26" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A26" s="19" t="s">
         <v>407</v>
       </c>
@@ -12780,7 +12780,7 @@
         <v>1322</v>
       </c>
     </row>
-    <row r="27" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="27" spans="1:5" s="10" customFormat="1" hidden="1">
       <c r="A27" s="19" t="s">
         <v>407</v>
       </c>
@@ -12814,7 +12814,7 @@
         <v>1326</v>
       </c>
     </row>
-    <row r="29" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="29" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A29" s="19" t="s">
         <v>407</v>
       </c>
@@ -12831,7 +12831,7 @@
         <v>1328</v>
       </c>
     </row>
-    <row r="30" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="30" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A30" s="19" t="s">
         <v>407</v>
       </c>
@@ -12848,7 +12848,7 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="31" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="31" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A31" s="19" t="s">
         <v>407</v>
       </c>
@@ -12865,7 +12865,7 @@
         <v>1332</v>
       </c>
     </row>
-    <row r="32" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="32" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A32" s="19" t="s">
         <v>407</v>
       </c>
@@ -12882,7 +12882,7 @@
         <v>1334</v>
       </c>
     </row>
-    <row r="33" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="33" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A33" s="19" t="s">
         <v>407</v>
       </c>
@@ -12899,7 +12899,7 @@
         <v>1336</v>
       </c>
     </row>
-    <row r="34" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="34" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A34" s="19" t="s">
         <v>407</v>
       </c>
@@ -12916,7 +12916,7 @@
         <v>1338</v>
       </c>
     </row>
-    <row r="35" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="35" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A35" s="19" t="s">
         <v>407</v>
       </c>
@@ -12950,7 +12950,7 @@
         <v>1342</v>
       </c>
     </row>
-    <row r="37" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="37" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A37" s="19" t="s">
         <v>407</v>
       </c>
@@ -12967,7 +12967,7 @@
         <v>1344</v>
       </c>
     </row>
-    <row r="38" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="38" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A38" s="19" t="s">
         <v>407</v>
       </c>
@@ -12984,7 +12984,7 @@
         <v>1346</v>
       </c>
     </row>
-    <row r="39" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="39" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A39" s="19" t="s">
         <v>407</v>
       </c>
@@ -13001,7 +13001,7 @@
         <v>1348</v>
       </c>
     </row>
-    <row r="40" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="40" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A40" s="19" t="s">
         <v>407</v>
       </c>
@@ -13018,7 +13018,7 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="41" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="41" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A41" s="19" t="s">
         <v>407</v>
       </c>
@@ -13035,7 +13035,7 @@
         <v>1352</v>
       </c>
     </row>
-    <row r="42" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="42" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A42" s="19" t="s">
         <v>407</v>
       </c>
@@ -13052,7 +13052,7 @@
         <v>1354</v>
       </c>
     </row>
-    <row r="43" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="43" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A43" s="19" t="s">
         <v>407</v>
       </c>
@@ -13069,7 +13069,7 @@
         <v>1356</v>
       </c>
     </row>
-    <row r="44" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="44" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A44" s="19" t="s">
         <v>407</v>
       </c>
@@ -13086,7 +13086,7 @@
         <v>1358</v>
       </c>
     </row>
-    <row r="45" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="45" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A45" s="19" t="s">
         <v>407</v>
       </c>
@@ -13120,7 +13120,7 @@
         <v>1362</v>
       </c>
     </row>
-    <row r="47" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="47" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A47" s="19" t="s">
         <v>407</v>
       </c>
@@ -13137,7 +13137,7 @@
         <v>1364</v>
       </c>
     </row>
-    <row r="48" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="48" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A48" s="19" t="s">
         <v>407</v>
       </c>
@@ -13154,7 +13154,7 @@
         <v>1366</v>
       </c>
     </row>
-    <row r="49" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="49" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A49" s="19" t="s">
         <v>407</v>
       </c>
@@ -13171,7 +13171,7 @@
         <v>1368</v>
       </c>
     </row>
-    <row r="50" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="50" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A50" s="19" t="s">
         <v>407</v>
       </c>
@@ -13188,7 +13188,7 @@
         <v>1370</v>
       </c>
     </row>
-    <row r="51" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="51" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A51" s="19" t="s">
         <v>407</v>
       </c>
@@ -13205,7 +13205,7 @@
         <v>1372</v>
       </c>
     </row>
-    <row r="52" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="52" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A52" s="19" t="s">
         <v>407</v>
       </c>
@@ -13222,7 +13222,7 @@
         <v>1374</v>
       </c>
     </row>
-    <row r="53" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="53" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A53" s="19" t="s">
         <v>407</v>
       </c>
@@ -13239,7 +13239,7 @@
         <v>1376</v>
       </c>
     </row>
-    <row r="54" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="54" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A54" s="19" t="s">
         <v>407</v>
       </c>
@@ -13256,7 +13256,7 @@
         <v>1378</v>
       </c>
     </row>
-    <row r="55" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="55" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A55" s="19" t="s">
         <v>407</v>
       </c>
@@ -13273,7 +13273,7 @@
         <v>1380</v>
       </c>
     </row>
-    <row r="56" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="56" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A56" s="19" t="s">
         <v>407</v>
       </c>
@@ -13290,7 +13290,7 @@
         <v>1382</v>
       </c>
     </row>
-    <row r="57" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="57" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A57" s="19" t="s">
         <v>407</v>
       </c>
@@ -13307,7 +13307,7 @@
         <v>1384</v>
       </c>
     </row>
-    <row r="58" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="58" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A58" s="19" t="s">
         <v>407</v>
       </c>
@@ -13324,7 +13324,7 @@
         <v>1386</v>
       </c>
     </row>
-    <row r="59" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="59" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A59" s="19" t="s">
         <v>407</v>
       </c>
@@ -13341,7 +13341,7 @@
         <v>1388</v>
       </c>
     </row>
-    <row r="60" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="60" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A60" s="19" t="s">
         <v>407</v>
       </c>
@@ -13358,7 +13358,7 @@
         <v>1390</v>
       </c>
     </row>
-    <row r="61" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="61" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A61" s="19" t="s">
         <v>407</v>
       </c>
@@ -13375,7 +13375,7 @@
         <v>1392</v>
       </c>
     </row>
-    <row r="62" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="62" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A62" s="19" t="s">
         <v>407</v>
       </c>
@@ -13392,7 +13392,7 @@
         <v>1394</v>
       </c>
     </row>
-    <row r="63" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="63" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A63" s="19" t="s">
         <v>407</v>
       </c>
@@ -13409,7 +13409,7 @@
         <v>1396</v>
       </c>
     </row>
-    <row r="64" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="64" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A64" s="19" t="s">
         <v>407</v>
       </c>
@@ -13426,7 +13426,7 @@
         <v>1398</v>
       </c>
     </row>
-    <row r="65" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="65" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A65" s="19" t="s">
         <v>407</v>
       </c>
@@ -13443,7 +13443,7 @@
         <v>1400</v>
       </c>
     </row>
-    <row r="66" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="66" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A66" s="19" t="s">
         <v>407</v>
       </c>
@@ -13460,7 +13460,7 @@
         <v>1402</v>
       </c>
     </row>
-    <row r="67" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="67" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A67" s="19" t="s">
         <v>407</v>
       </c>
@@ -13477,7 +13477,7 @@
         <v>1404</v>
       </c>
     </row>
-    <row r="68" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="68" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A68" s="19" t="s">
         <v>407</v>
       </c>
@@ -13494,7 +13494,7 @@
         <v>1406</v>
       </c>
     </row>
-    <row r="69" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="69" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A69" s="19" t="s">
         <v>407</v>
       </c>
@@ -13511,7 +13511,7 @@
         <v>1408</v>
       </c>
     </row>
-    <row r="70" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="70" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A70" s="19" t="s">
         <v>407</v>
       </c>
@@ -13528,7 +13528,7 @@
         <v>1410</v>
       </c>
     </row>
-    <row r="71" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="71" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A71" s="19" t="s">
         <v>407</v>
       </c>
@@ -13545,7 +13545,7 @@
         <v>1412</v>
       </c>
     </row>
-    <row r="72" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="72" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A72" s="19" t="s">
         <v>407</v>
       </c>
@@ -13562,7 +13562,7 @@
         <v>1414</v>
       </c>
     </row>
-    <row r="73" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="73" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A73" s="19" t="s">
         <v>407</v>
       </c>
@@ -13579,7 +13579,7 @@
         <v>1416</v>
       </c>
     </row>
-    <row r="74" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="74" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A74" s="19" t="s">
         <v>407</v>
       </c>
@@ -13596,7 +13596,7 @@
         <v>1418</v>
       </c>
     </row>
-    <row r="75" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="75" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A75" s="19" t="s">
         <v>407</v>
       </c>
@@ -13613,7 +13613,7 @@
         <v>1420</v>
       </c>
     </row>
-    <row r="76" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="76" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A76" s="19" t="s">
         <v>407</v>
       </c>
@@ -13630,7 +13630,7 @@
         <v>1422</v>
       </c>
     </row>
-    <row r="77" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="77" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A77" s="19" t="s">
         <v>407</v>
       </c>
@@ -13647,7 +13647,7 @@
         <v>1424</v>
       </c>
     </row>
-    <row r="78" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="78" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A78" s="19" t="s">
         <v>407</v>
       </c>
@@ -13715,7 +13715,7 @@
         <v>1432</v>
       </c>
     </row>
-    <row r="82" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="82" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A82" s="19" t="s">
         <v>407</v>
       </c>
@@ -13732,7 +13732,7 @@
         <v>1434</v>
       </c>
     </row>
-    <row r="83" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="83" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A83" s="19" t="s">
         <v>407</v>
       </c>
@@ -13749,7 +13749,7 @@
         <v>1436</v>
       </c>
     </row>
-    <row r="84" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="84" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A84" s="19" t="s">
         <v>407</v>
       </c>
@@ -13783,7 +13783,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="86" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="86" spans="1:5" s="10" customFormat="1" hidden="1">
       <c r="A86" s="19" t="s">
         <v>407</v>
       </c>
@@ -13800,7 +13800,7 @@
         <v>1442</v>
       </c>
     </row>
-    <row r="87" spans="1:5" s="10" customFormat="1" ht="29">
+    <row r="87" spans="1:5" s="10" customFormat="1" ht="28.8">
       <c r="A87" s="19" t="s">
         <v>407</v>
       </c>
@@ -13817,7 +13817,7 @@
         <v>1444</v>
       </c>
     </row>
-    <row r="88" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="88" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A88" s="19" t="s">
         <v>407</v>
       </c>
@@ -13834,7 +13834,7 @@
         <v>1446</v>
       </c>
     </row>
-    <row r="89" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="89" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A89" s="19" t="s">
         <v>407</v>
       </c>
@@ -13851,7 +13851,7 @@
         <v>1448</v>
       </c>
     </row>
-    <row r="90" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="90" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A90" s="19" t="s">
         <v>407</v>
       </c>
@@ -13868,7 +13868,7 @@
         <v>1450</v>
       </c>
     </row>
-    <row r="91" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="91" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A91" s="19" t="s">
         <v>407</v>
       </c>
@@ -13902,7 +13902,7 @@
         <v>1454</v>
       </c>
     </row>
-    <row r="93" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="93" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A93" s="19" t="s">
         <v>407</v>
       </c>
@@ -13936,7 +13936,7 @@
         <v>1458</v>
       </c>
     </row>
-    <row r="95" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="95" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A95" s="19" t="s">
         <v>407</v>
       </c>
@@ -13953,7 +13953,7 @@
         <v>1460</v>
       </c>
     </row>
-    <row r="96" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="96" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A96" s="19" t="s">
         <v>407</v>
       </c>
@@ -13970,7 +13970,7 @@
         <v>1462</v>
       </c>
     </row>
-    <row r="97" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="97" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A97" s="19" t="s">
         <v>407</v>
       </c>
@@ -13987,7 +13987,7 @@
         <v>1464</v>
       </c>
     </row>
-    <row r="98" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="98" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A98" s="19" t="s">
         <v>407</v>
       </c>
@@ -14004,7 +14004,7 @@
         <v>1466</v>
       </c>
     </row>
-    <row r="99" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="99" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A99" s="19" t="s">
         <v>407</v>
       </c>
@@ -14021,7 +14021,7 @@
         <v>1468</v>
       </c>
     </row>
-    <row r="100" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="100" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A100" s="19" t="s">
         <v>407</v>
       </c>
@@ -14055,7 +14055,7 @@
         <v>1472</v>
       </c>
     </row>
-    <row r="102" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="102" spans="1:5" s="10" customFormat="1" hidden="1">
       <c r="A102" s="19" t="s">
         <v>407</v>
       </c>
@@ -14089,7 +14089,7 @@
         <v>1476</v>
       </c>
     </row>
-    <row r="104" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="104" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A104" s="19" t="s">
         <v>407</v>
       </c>
@@ -14106,7 +14106,7 @@
         <v>1478</v>
       </c>
     </row>
-    <row r="105" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="105" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A105" s="19" t="s">
         <v>407</v>
       </c>
@@ -14123,7 +14123,7 @@
         <v>1480</v>
       </c>
     </row>
-    <row r="106" spans="1:5" s="10" customFormat="1" ht="43.5" hidden="1">
+    <row r="106" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A106" s="19" t="s">
         <v>407</v>
       </c>
@@ -14140,7 +14140,7 @@
         <v>1482</v>
       </c>
     </row>
-    <row r="107" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="107" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A107" s="19" t="s">
         <v>407</v>
       </c>
@@ -14157,7 +14157,7 @@
         <v>1484</v>
       </c>
     </row>
-    <row r="108" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="108" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A108" s="19" t="s">
         <v>407</v>
       </c>
@@ -14174,7 +14174,7 @@
         <v>1486</v>
       </c>
     </row>
-    <row r="109" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="109" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A109" s="19" t="s">
         <v>407</v>
       </c>
@@ -14191,7 +14191,7 @@
         <v>1488</v>
       </c>
     </row>
-    <row r="110" spans="1:5" s="10" customFormat="1" ht="43.5" hidden="1">
+    <row r="110" spans="1:5" s="10" customFormat="1" ht="43.2" hidden="1">
       <c r="A110" s="19" t="s">
         <v>407</v>
       </c>
@@ -14208,7 +14208,7 @@
         <v>1490</v>
       </c>
     </row>
-    <row r="111" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="111" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A111" s="19" t="s">
         <v>407</v>
       </c>
@@ -14225,7 +14225,7 @@
         <v>1492</v>
       </c>
     </row>
-    <row r="112" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="112" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A112" s="19" t="s">
         <v>407</v>
       </c>
@@ -14242,7 +14242,7 @@
         <v>1494</v>
       </c>
     </row>
-    <row r="113" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="113" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A113" s="19" t="s">
         <v>407</v>
       </c>
@@ -14259,7 +14259,7 @@
         <v>1496</v>
       </c>
     </row>
-    <row r="114" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="114" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A114" s="19" t="s">
         <v>407</v>
       </c>
@@ -14276,7 +14276,7 @@
         <v>1498</v>
       </c>
     </row>
-    <row r="115" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="115" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A115" s="19" t="s">
         <v>407</v>
       </c>
@@ -14293,7 +14293,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="116" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="116" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A116" s="19" t="s">
         <v>407</v>
       </c>
@@ -14310,7 +14310,7 @@
         <v>1502</v>
       </c>
     </row>
-    <row r="117" spans="1:5" s="10" customFormat="1" ht="43.5" hidden="1">
+    <row r="117" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A117" s="19" t="s">
         <v>407</v>
       </c>
@@ -14327,7 +14327,7 @@
         <v>1504</v>
       </c>
     </row>
-    <row r="118" spans="1:5" s="10" customFormat="1" ht="43.5" hidden="1">
+    <row r="118" spans="1:5" s="10" customFormat="1" ht="43.2" hidden="1">
       <c r="A118" s="19" t="s">
         <v>407</v>
       </c>
@@ -14344,7 +14344,7 @@
         <v>1506</v>
       </c>
     </row>
-    <row r="119" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="119" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A119" s="19" t="s">
         <v>407</v>
       </c>
@@ -14361,7 +14361,7 @@
         <v>1508</v>
       </c>
     </row>
-    <row r="120" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="120" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A120" s="19" t="s">
         <v>407</v>
       </c>
@@ -14378,7 +14378,7 @@
         <v>1510</v>
       </c>
     </row>
-    <row r="121" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="121" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A121" s="19" t="s">
         <v>407</v>
       </c>
@@ -14395,7 +14395,7 @@
         <v>1512</v>
       </c>
     </row>
-    <row r="122" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="122" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A122" s="19" t="s">
         <v>407</v>
       </c>
@@ -14412,7 +14412,7 @@
         <v>1514</v>
       </c>
     </row>
-    <row r="123" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="123" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A123" s="19" t="s">
         <v>407</v>
       </c>
@@ -14429,7 +14429,7 @@
         <v>1516</v>
       </c>
     </row>
-    <row r="124" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="124" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A124" s="19" t="s">
         <v>407</v>
       </c>
@@ -14497,7 +14497,7 @@
         <v>1524</v>
       </c>
     </row>
-    <row r="128" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="128" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A128" s="19" t="s">
         <v>407</v>
       </c>
@@ -14514,7 +14514,7 @@
         <v>1526</v>
       </c>
     </row>
-    <row r="129" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="129" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A129" s="19" t="s">
         <v>407</v>
       </c>
@@ -14531,7 +14531,7 @@
         <v>1528</v>
       </c>
     </row>
-    <row r="130" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="130" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A130" s="19" t="s">
         <v>407</v>
       </c>
@@ -14548,7 +14548,7 @@
         <v>1530</v>
       </c>
     </row>
-    <row r="131" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="131" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A131" s="19" t="s">
         <v>407</v>
       </c>
@@ -14565,7 +14565,7 @@
         <v>1532</v>
       </c>
     </row>
-    <row r="132" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="132" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A132" s="19" t="s">
         <v>407</v>
       </c>
@@ -14599,7 +14599,7 @@
         <v>1536</v>
       </c>
     </row>
-    <row r="134" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="134" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A134" s="19" t="s">
         <v>407</v>
       </c>
@@ -14616,7 +14616,7 @@
         <v>1538</v>
       </c>
     </row>
-    <row r="135" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="135" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A135" s="19" t="s">
         <v>407</v>
       </c>
@@ -14633,7 +14633,7 @@
         <v>1540</v>
       </c>
     </row>
-    <row r="136" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="136" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A136" s="19" t="s">
         <v>407</v>
       </c>
@@ -14667,7 +14667,7 @@
         <v>1544</v>
       </c>
     </row>
-    <row r="138" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="138" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A138" s="19" t="s">
         <v>407</v>
       </c>
@@ -14684,7 +14684,7 @@
         <v>1546</v>
       </c>
     </row>
-    <row r="139" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="139" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A139" s="19" t="s">
         <v>407</v>
       </c>
@@ -14701,7 +14701,7 @@
         <v>1548</v>
       </c>
     </row>
-    <row r="140" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="140" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A140" s="19" t="s">
         <v>407</v>
       </c>
@@ -14718,7 +14718,7 @@
         <v>1550</v>
       </c>
     </row>
-    <row r="141" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="141" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A141" s="19" t="s">
         <v>407</v>
       </c>
@@ -14735,7 +14735,7 @@
         <v>1552</v>
       </c>
     </row>
-    <row r="142" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="142" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A142" s="19" t="s">
         <v>407</v>
       </c>
@@ -14752,7 +14752,7 @@
         <v>1554</v>
       </c>
     </row>
-    <row r="143" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="143" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A143" s="19" t="s">
         <v>407</v>
       </c>
@@ -14769,7 +14769,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="144" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="144" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A144" s="19" t="s">
         <v>407</v>
       </c>
@@ -14786,7 +14786,7 @@
         <v>1558</v>
       </c>
     </row>
-    <row r="145" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="145" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A145" s="19" t="s">
         <v>407</v>
       </c>
@@ -14820,7 +14820,7 @@
         <v>1562</v>
       </c>
     </row>
-    <row r="147" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="147" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A147" s="19" t="s">
         <v>407</v>
       </c>
@@ -14837,7 +14837,7 @@
         <v>1564</v>
       </c>
     </row>
-    <row r="148" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="148" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A148" s="19" t="s">
         <v>407</v>
       </c>
@@ -14854,7 +14854,7 @@
         <v>1566</v>
       </c>
     </row>
-    <row r="149" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="149" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A149" s="19" t="s">
         <v>407</v>
       </c>
@@ -14871,7 +14871,7 @@
         <v>1568</v>
       </c>
     </row>
-    <row r="150" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="150" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A150" s="19" t="s">
         <v>407</v>
       </c>
@@ -14888,7 +14888,7 @@
         <v>1570</v>
       </c>
     </row>
-    <row r="151" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="151" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A151" s="19" t="s">
         <v>407</v>
       </c>
@@ -14905,7 +14905,7 @@
         <v>1572</v>
       </c>
     </row>
-    <row r="152" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="152" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A152" s="19" t="s">
         <v>407</v>
       </c>
@@ -14922,7 +14922,7 @@
         <v>1574</v>
       </c>
     </row>
-    <row r="153" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="153" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A153" s="19" t="s">
         <v>407</v>
       </c>
@@ -14956,7 +14956,7 @@
         <v>1578</v>
       </c>
     </row>
-    <row r="155" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="155" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A155" s="19" t="s">
         <v>407</v>
       </c>
@@ -14973,7 +14973,7 @@
         <v>1580</v>
       </c>
     </row>
-    <row r="156" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="156" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A156" s="19" t="s">
         <v>407</v>
       </c>
@@ -14990,7 +14990,7 @@
         <v>1582</v>
       </c>
     </row>
-    <row r="157" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="157" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A157" s="19" t="s">
         <v>407</v>
       </c>
@@ -15007,7 +15007,7 @@
         <v>1584</v>
       </c>
     </row>
-    <row r="158" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="158" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A158" s="19" t="s">
         <v>407</v>
       </c>
@@ -15024,7 +15024,7 @@
         <v>1586</v>
       </c>
     </row>
-    <row r="159" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="159" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A159" s="19" t="s">
         <v>407</v>
       </c>
@@ -15041,7 +15041,7 @@
         <v>1588</v>
       </c>
     </row>
-    <row r="160" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="160" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A160" s="19" t="s">
         <v>407</v>
       </c>
@@ -15058,7 +15058,7 @@
         <v>1590</v>
       </c>
     </row>
-    <row r="161" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="161" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A161" s="19" t="s">
         <v>407</v>
       </c>
@@ -15075,7 +15075,7 @@
         <v>1592</v>
       </c>
     </row>
-    <row r="162" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="162" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A162" s="19" t="s">
         <v>407</v>
       </c>
@@ -15092,7 +15092,7 @@
         <v>1594</v>
       </c>
     </row>
-    <row r="163" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="163" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A163" s="19" t="s">
         <v>407</v>
       </c>
@@ -15109,7 +15109,7 @@
         <v>1596</v>
       </c>
     </row>
-    <row r="164" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="164" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A164" s="19" t="s">
         <v>407</v>
       </c>
@@ -15126,7 +15126,7 @@
         <v>1598</v>
       </c>
     </row>
-    <row r="165" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="165" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A165" s="19" t="s">
         <v>407</v>
       </c>
@@ -15143,7 +15143,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="166" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="166" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A166" s="19" t="s">
         <v>407</v>
       </c>
@@ -15160,7 +15160,7 @@
         <v>1602</v>
       </c>
     </row>
-    <row r="167" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="167" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A167" s="19" t="s">
         <v>407</v>
       </c>
@@ -15177,7 +15177,7 @@
         <v>1604</v>
       </c>
     </row>
-    <row r="168" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="168" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A168" s="19" t="s">
         <v>407</v>
       </c>
@@ -15194,7 +15194,7 @@
         <v>1606</v>
       </c>
     </row>
-    <row r="169" spans="1:5" s="10" customFormat="1" ht="43.5" hidden="1">
+    <row r="169" spans="1:5" s="10" customFormat="1" ht="43.2" hidden="1">
       <c r="A169" s="19" t="s">
         <v>407</v>
       </c>
@@ -15211,7 +15211,7 @@
         <v>1608</v>
       </c>
     </row>
-    <row r="170" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="170" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A170" s="19" t="s">
         <v>407</v>
       </c>
@@ -15228,7 +15228,7 @@
         <v>1610</v>
       </c>
     </row>
-    <row r="171" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="171" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A171" s="19" t="s">
         <v>407</v>
       </c>
@@ -15245,7 +15245,7 @@
         <v>1612</v>
       </c>
     </row>
-    <row r="172" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="172" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A172" s="19" t="s">
         <v>407</v>
       </c>
@@ -15262,7 +15262,7 @@
         <v>1614</v>
       </c>
     </row>
-    <row r="173" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="173" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A173" s="19" t="s">
         <v>407</v>
       </c>
@@ -15279,7 +15279,7 @@
         <v>1616</v>
       </c>
     </row>
-    <row r="174" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="174" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A174" s="19" t="s">
         <v>407</v>
       </c>
@@ -15313,7 +15313,7 @@
         <v>1620</v>
       </c>
     </row>
-    <row r="176" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="176" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A176" s="19" t="s">
         <v>407</v>
       </c>
@@ -15330,7 +15330,7 @@
         <v>1622</v>
       </c>
     </row>
-    <row r="177" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="177" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A177" s="19" t="s">
         <v>407</v>
       </c>
@@ -15347,7 +15347,7 @@
         <v>1624</v>
       </c>
     </row>
-    <row r="178" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="178" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A178" s="19" t="s">
         <v>407</v>
       </c>
@@ -15364,7 +15364,7 @@
         <v>1626</v>
       </c>
     </row>
-    <row r="179" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="179" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A179" s="19" t="s">
         <v>407</v>
       </c>
@@ -15381,7 +15381,7 @@
         <v>1628</v>
       </c>
     </row>
-    <row r="180" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="180" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A180" s="19" t="s">
         <v>407</v>
       </c>
@@ -15398,7 +15398,7 @@
         <v>1630</v>
       </c>
     </row>
-    <row r="181" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="181" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A181" s="19" t="s">
         <v>407</v>
       </c>
@@ -15415,7 +15415,7 @@
         <v>1632</v>
       </c>
     </row>
-    <row r="182" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="182" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A182" s="19" t="s">
         <v>407</v>
       </c>
@@ -15432,7 +15432,7 @@
         <v>1634</v>
       </c>
     </row>
-    <row r="183" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="183" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A183" s="19" t="s">
         <v>407</v>
       </c>
@@ -15449,7 +15449,7 @@
         <v>1636</v>
       </c>
     </row>
-    <row r="184" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="184" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A184" s="19" t="s">
         <v>407</v>
       </c>
@@ -15466,7 +15466,7 @@
         <v>1638</v>
       </c>
     </row>
-    <row r="185" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="185" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A185" s="19" t="s">
         <v>407</v>
       </c>
@@ -15483,7 +15483,7 @@
         <v>1640</v>
       </c>
     </row>
-    <row r="186" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="186" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A186" s="19" t="s">
         <v>407</v>
       </c>
@@ -15500,7 +15500,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="187" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="187" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A187" s="19" t="s">
         <v>407</v>
       </c>
@@ -15534,7 +15534,7 @@
         <v>1646</v>
       </c>
     </row>
-    <row r="189" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="189" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A189" s="19" t="s">
         <v>407</v>
       </c>
@@ -15551,7 +15551,7 @@
         <v>1648</v>
       </c>
     </row>
-    <row r="190" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="190" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A190" s="19" t="s">
         <v>407</v>
       </c>
@@ -15585,7 +15585,7 @@
         <v>1652</v>
       </c>
     </row>
-    <row r="192" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="192" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A192" s="19" t="s">
         <v>407</v>
       </c>
@@ -15602,7 +15602,7 @@
         <v>1654</v>
       </c>
     </row>
-    <row r="193" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="193" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A193" s="19" t="s">
         <v>407</v>
       </c>
@@ -15619,7 +15619,7 @@
         <v>1656</v>
       </c>
     </row>
-    <row r="194" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="194" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A194" s="19" t="s">
         <v>407</v>
       </c>
@@ -15636,7 +15636,7 @@
         <v>1658</v>
       </c>
     </row>
-    <row r="195" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="195" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A195" s="19" t="s">
         <v>407</v>
       </c>
@@ -15653,7 +15653,7 @@
         <v>1660</v>
       </c>
     </row>
-    <row r="196" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="196" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A196" s="19" t="s">
         <v>407</v>
       </c>
@@ -15670,7 +15670,7 @@
         <v>1662</v>
       </c>
     </row>
-    <row r="197" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="197" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A197" s="19" t="s">
         <v>407</v>
       </c>
@@ -15687,7 +15687,7 @@
         <v>1664</v>
       </c>
     </row>
-    <row r="198" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="198" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A198" s="19" t="s">
         <v>407</v>
       </c>
@@ -15721,7 +15721,7 @@
         <v>1668</v>
       </c>
     </row>
-    <row r="200" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="200" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A200" s="19" t="s">
         <v>407</v>
       </c>
@@ -15755,7 +15755,7 @@
         <v>1672</v>
       </c>
     </row>
-    <row r="202" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="202" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A202" s="19" t="s">
         <v>407</v>
       </c>
@@ -15772,7 +15772,7 @@
         <v>1674</v>
       </c>
     </row>
-    <row r="203" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="203" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A203" s="19" t="s">
         <v>407</v>
       </c>
@@ -15789,7 +15789,7 @@
         <v>1676</v>
       </c>
     </row>
-    <row r="204" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="204" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A204" s="19" t="s">
         <v>407</v>
       </c>
@@ -15806,7 +15806,7 @@
         <v>1678</v>
       </c>
     </row>
-    <row r="205" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="205" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A205" s="19" t="s">
         <v>407</v>
       </c>
@@ -15823,7 +15823,7 @@
         <v>1680</v>
       </c>
     </row>
-    <row r="206" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="206" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A206" s="19" t="s">
         <v>407</v>
       </c>
@@ -15840,7 +15840,7 @@
         <v>1682</v>
       </c>
     </row>
-    <row r="207" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="207" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A207" s="19" t="s">
         <v>407</v>
       </c>
@@ -15857,7 +15857,7 @@
         <v>1684</v>
       </c>
     </row>
-    <row r="208" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="208" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A208" s="19" t="s">
         <v>407</v>
       </c>
@@ -15874,7 +15874,7 @@
         <v>1686</v>
       </c>
     </row>
-    <row r="209" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="209" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A209" s="19" t="s">
         <v>407</v>
       </c>
@@ -15891,7 +15891,7 @@
         <v>1688</v>
       </c>
     </row>
-    <row r="210" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="210" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A210" s="19" t="s">
         <v>407</v>
       </c>
@@ -15925,7 +15925,7 @@
         <v>1692</v>
       </c>
     </row>
-    <row r="212" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="212" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A212" s="19" t="s">
         <v>407</v>
       </c>
@@ -15942,7 +15942,7 @@
         <v>1694</v>
       </c>
     </row>
-    <row r="213" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="213" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A213" s="19" t="s">
         <v>407</v>
       </c>
@@ -15993,7 +15993,7 @@
         <v>1700</v>
       </c>
     </row>
-    <row r="216" spans="1:5" s="10" customFormat="1" ht="43.5" hidden="1">
+    <row r="216" spans="1:5" s="10" customFormat="1" ht="43.2" hidden="1">
       <c r="A216" s="19" t="s">
         <v>407</v>
       </c>
@@ -16010,7 +16010,7 @@
         <v>1702</v>
       </c>
     </row>
-    <row r="217" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="217" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A217" s="19" t="s">
         <v>407</v>
       </c>
@@ -16044,7 +16044,7 @@
         <v>1706</v>
       </c>
     </row>
-    <row r="219" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="219" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A219" s="19" t="s">
         <v>407</v>
       </c>
@@ -16061,7 +16061,7 @@
         <v>1708</v>
       </c>
     </row>
-    <row r="220" spans="1:5" s="10" customFormat="1" ht="29" hidden="1">
+    <row r="220" spans="1:5" s="10" customFormat="1" ht="28.8" hidden="1">
       <c r="A220" s="19" t="s">
         <v>407</v>
       </c>
@@ -16345,24 +16345,25 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8D30C07-B92F-494E-AD16-8F2C62A91261}">
   <dimension ref="A1:L56"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="25.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" customWidth="1"/>
+    <col min="4" max="4" width="26.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" t="s">
-        <v>1780</v>
+        <v>1874</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>1875</v>
       </c>
       <c r="C1" t="s">
-        <v>66</v>
+        <v>1877</v>
       </c>
       <c r="D1" t="s">
-        <v>1779</v>
+        <v>1878</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -16793,7 +16794,7 @@
         <v>540</v>
       </c>
       <c r="B32" t="s">
-        <v>1816</v>
+        <v>1813</v>
       </c>
       <c r="C32" t="s">
         <v>542</v>
@@ -17149,26 +17150,26 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{547CAAEB-A403-45F4-B122-C4489DDB4C52}">
   <dimension ref="A1:D60"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="7.6328125" customWidth="1"/>
-    <col min="2" max="2" width="25.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.6328125" customWidth="1"/>
-    <col min="4" max="4" width="26.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" customWidth="1"/>
+    <col min="2" max="2" width="25.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.6640625" customWidth="1"/>
+    <col min="4" max="4" width="26.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>1780</v>
+        <v>1874</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>1875</v>
       </c>
       <c r="C1" t="s">
-        <v>1132</v>
+        <v>1877</v>
       </c>
       <c r="D1" t="s">
-        <v>1817</v>
+        <v>1878</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -17207,7 +17208,7 @@
         <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>1781</v>
+        <v>1778</v>
       </c>
       <c r="D4" t="s">
         <v>417</v>
@@ -17221,10 +17222,10 @@
         <v>130</v>
       </c>
       <c r="C5" t="s">
-        <v>1782</v>
+        <v>1779</v>
       </c>
       <c r="D5" t="s">
-        <v>1783</v>
+        <v>1780</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -17235,7 +17236,7 @@
         <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>1784</v>
+        <v>1781</v>
       </c>
       <c r="D6" t="s">
         <v>421</v>
@@ -17249,7 +17250,7 @@
         <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>1785</v>
+        <v>1782</v>
       </c>
       <c r="D7" t="s">
         <v>38</v>
@@ -17263,7 +17264,7 @@
         <v>49</v>
       </c>
       <c r="C8" t="s">
-        <v>1786</v>
+        <v>1783</v>
       </c>
       <c r="D8" t="s">
         <v>49</v>
@@ -17277,7 +17278,7 @@
         <v>51</v>
       </c>
       <c r="C9" t="s">
-        <v>1787</v>
+        <v>1784</v>
       </c>
       <c r="D9" t="s">
         <v>51</v>
@@ -17333,7 +17334,7 @@
         <v>47</v>
       </c>
       <c r="C13" t="s">
-        <v>1788</v>
+        <v>1785</v>
       </c>
       <c r="D13" t="s">
         <v>432</v>
@@ -17361,10 +17362,10 @@
         <v>27</v>
       </c>
       <c r="C15" t="s">
-        <v>1789</v>
+        <v>1786</v>
       </c>
       <c r="D15" t="s">
-        <v>1790</v>
+        <v>1787</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -17459,10 +17460,10 @@
         <v>452</v>
       </c>
       <c r="C22" t="s">
-        <v>1791</v>
+        <v>1788</v>
       </c>
       <c r="D22" t="s">
-        <v>1792</v>
+        <v>1789</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -17473,10 +17474,10 @@
         <v>23</v>
       </c>
       <c r="C23" t="s">
-        <v>1793</v>
+        <v>1790</v>
       </c>
       <c r="D23" t="s">
-        <v>1794</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -17831,86 +17832,86 @@
     </row>
     <row r="49" spans="1:4">
       <c r="A49" t="s">
+        <v>1792</v>
+      </c>
+      <c r="B49" t="s">
+        <v>1793</v>
+      </c>
+      <c r="C49" t="s">
+        <v>1794</v>
+      </c>
+      <c r="D49" t="s">
         <v>1795</v>
-      </c>
-      <c r="B49" t="s">
-        <v>1796</v>
-      </c>
-      <c r="C49" t="s">
-        <v>1797</v>
-      </c>
-      <c r="D49" t="s">
-        <v>1798</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" t="s">
-        <v>1799</v>
+        <v>1796</v>
       </c>
       <c r="B50" t="s">
-        <v>1800</v>
+        <v>1797</v>
       </c>
       <c r="C50" t="s">
-        <v>1801</v>
+        <v>1798</v>
       </c>
       <c r="D50" t="s">
-        <v>1800</v>
+        <v>1797</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" t="s">
-        <v>1802</v>
+        <v>1799</v>
       </c>
       <c r="B51" t="s">
-        <v>1803</v>
+        <v>1800</v>
       </c>
       <c r="C51" t="s">
-        <v>1804</v>
+        <v>1801</v>
       </c>
       <c r="D51" t="s">
-        <v>1803</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" t="s">
-        <v>1805</v>
+        <v>1802</v>
       </c>
       <c r="B52" t="s">
-        <v>1806</v>
+        <v>1803</v>
       </c>
       <c r="C52" t="s">
-        <v>1807</v>
+        <v>1804</v>
       </c>
       <c r="D52" t="s">
-        <v>1806</v>
+        <v>1803</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" t="s">
-        <v>1808</v>
+        <v>1805</v>
       </c>
       <c r="B53" t="s">
-        <v>1809</v>
+        <v>1806</v>
       </c>
       <c r="C53" t="s">
-        <v>1810</v>
+        <v>1807</v>
       </c>
       <c r="D53" t="s">
-        <v>1809</v>
+        <v>1806</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" t="s">
+        <v>1808</v>
+      </c>
+      <c r="B54" t="s">
+        <v>1809</v>
+      </c>
+      <c r="C54" t="s">
+        <v>1810</v>
+      </c>
+      <c r="D54" t="s">
         <v>1811</v>
-      </c>
-      <c r="B54" t="s">
-        <v>1812</v>
-      </c>
-      <c r="C54" t="s">
-        <v>1813</v>
-      </c>
-      <c r="D54" t="s">
-        <v>1814</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -17921,7 +17922,7 @@
         <v>545</v>
       </c>
       <c r="C55" t="s">
-        <v>1815</v>
+        <v>1812</v>
       </c>
       <c r="D55" t="s">
         <v>547</v>
@@ -18008,13 +18009,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{617E1E86-4318-4373-98CB-6362DB1DB101}">
   <dimension ref="A1:I763"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="26.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="5" max="5" width="27.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.88671875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -39300,9 +39301,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF0433E0-5026-4073-87CF-A04A4E545664}">
   <dimension ref="A1:A11"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="12.7265625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="12.77734375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
@@ -39369,65 +39370,65 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10DEA558-E42D-42C7-87E1-199497B49C2E}">
   <dimension ref="A1:D29"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="17.453125" customWidth="1"/>
-    <col min="2" max="2" width="18.1796875" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" customWidth="1"/>
-    <col min="4" max="4" width="27.26953125" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="2" max="2" width="18.21875" customWidth="1"/>
+    <col min="3" max="3" width="12.21875" customWidth="1"/>
+    <col min="4" max="4" width="27.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
-        <v>1830</v>
+        <v>1826</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>1831</v>
+        <v>1827</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>1877</v>
+        <v>1873</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>1832</v>
+        <v>1828</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="42" t="s">
-        <v>1833</v>
+        <v>1829</v>
       </c>
       <c r="B2" s="42" t="s">
-        <v>1833</v>
+        <v>1829</v>
       </c>
       <c r="C2" s="42" t="s">
-        <v>1833</v>
+        <v>1829</v>
       </c>
       <c r="D2" s="42" t="s">
-        <v>1834</v>
+        <v>1830</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="4" t="s">
-        <v>1835</v>
+        <v>1831</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>1835</v>
+        <v>1831</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>1835</v>
+        <v>1831</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>1834</v>
+        <v>1830</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="42" t="s">
-        <v>1836</v>
+        <v>1832</v>
       </c>
       <c r="B4" s="42" t="s">
-        <v>1836</v>
+        <v>1832</v>
       </c>
       <c r="C4" s="42" t="s">
-        <v>1821</v>
+        <v>1817</v>
       </c>
       <c r="D4" s="42" t="s">
         <v>1737</v>
@@ -39435,27 +39436,27 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="4" t="s">
-        <v>1837</v>
+        <v>1833</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>1837</v>
+        <v>1833</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>1837</v>
+        <v>1833</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>1838</v>
+        <v>1834</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="42" t="s">
-        <v>1839</v>
+        <v>1835</v>
       </c>
       <c r="B6" s="42" t="s">
-        <v>1839</v>
+        <v>1835</v>
       </c>
       <c r="C6" s="42" t="s">
-        <v>1820</v>
+        <v>1816</v>
       </c>
       <c r="D6" s="42" t="s">
         <v>1732</v>
@@ -39463,13 +39464,13 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="4" t="s">
-        <v>1840</v>
+        <v>1836</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>1839</v>
+        <v>1835</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>1818</v>
+        <v>1814</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>1739</v>
@@ -39477,13 +39478,13 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="42" t="s">
-        <v>1841</v>
+        <v>1837</v>
       </c>
       <c r="B8" s="42" t="s">
-        <v>1839</v>
+        <v>1835</v>
       </c>
       <c r="C8" s="42" t="s">
-        <v>1827</v>
+        <v>1823</v>
       </c>
       <c r="D8" s="42" t="s">
         <v>1738</v>
@@ -39491,10 +39492,10 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="4" t="s">
-        <v>1842</v>
+        <v>1838</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>1839</v>
+        <v>1835</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>7</v>
@@ -39505,13 +39506,13 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="42" t="s">
-        <v>1843</v>
+        <v>1839</v>
       </c>
       <c r="B10" s="42" t="s">
-        <v>1843</v>
+        <v>1839</v>
       </c>
       <c r="C10" s="42" t="s">
-        <v>1828</v>
+        <v>1824</v>
       </c>
       <c r="D10" s="42" t="s">
         <v>1736</v>
@@ -39519,41 +39520,41 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="4" t="s">
-        <v>1844</v>
+        <v>1840</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>1843</v>
+        <v>1839</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>1845</v>
+        <v>1841</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>1846</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="42" t="s">
-        <v>1847</v>
+        <v>1843</v>
       </c>
       <c r="B12" s="42" t="s">
-        <v>1847</v>
+        <v>1843</v>
       </c>
       <c r="C12" s="42" t="s">
-        <v>1847</v>
+        <v>1843</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>1848</v>
+        <v>1844</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="4" t="s">
-        <v>1849</v>
+        <v>1845</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>1849</v>
+        <v>1845</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>1822</v>
+        <v>1818</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>1733</v>
@@ -39561,27 +39562,27 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="42" t="s">
-        <v>1850</v>
+        <v>1846</v>
       </c>
       <c r="B14" s="42" t="s">
-        <v>1849</v>
+        <v>1845</v>
       </c>
       <c r="C14" s="42" t="s">
-        <v>1851</v>
+        <v>1847</v>
       </c>
       <c r="D14" s="42" t="s">
-        <v>1852</v>
+        <v>1848</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="4" t="s">
-        <v>1853</v>
+        <v>1849</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>1849</v>
+        <v>1845</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>1829</v>
+        <v>1825</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>1741</v>
@@ -39589,10 +39590,10 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="42" t="s">
-        <v>1854</v>
+        <v>1850</v>
       </c>
       <c r="B16" s="42" t="s">
-        <v>1849</v>
+        <v>1845</v>
       </c>
       <c r="C16" s="42" t="s">
         <v>948</v>
@@ -39603,41 +39604,41 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="4" t="s">
-        <v>1855</v>
+        <v>1851</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>1855</v>
+        <v>1851</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>1856</v>
+        <v>1852</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>1857</v>
+        <v>1853</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="42" t="s">
-        <v>1858</v>
+        <v>1854</v>
       </c>
       <c r="B18" s="42" t="s">
-        <v>1858</v>
+        <v>1854</v>
       </c>
       <c r="C18" s="42" t="s">
-        <v>1859</v>
+        <v>1855</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>1860</v>
+        <v>1856</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="4" t="s">
-        <v>1861</v>
+        <v>1857</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>1861</v>
+        <v>1857</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>1823</v>
+        <v>1819</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>1735</v>
@@ -39645,27 +39646,27 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="42" t="s">
-        <v>1862</v>
+        <v>1858</v>
       </c>
       <c r="B20" s="42" t="s">
-        <v>1862</v>
+        <v>1858</v>
       </c>
       <c r="C20" s="42" t="s">
-        <v>1863</v>
+        <v>1859</v>
       </c>
       <c r="D20" s="42" t="s">
-        <v>1864</v>
+        <v>1860</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="4" t="s">
-        <v>1865</v>
+        <v>1861</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>1865</v>
+        <v>1861</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>1824</v>
+        <v>1820</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>1742</v>
@@ -39673,41 +39674,41 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="42" t="s">
-        <v>1866</v>
+        <v>1862</v>
       </c>
       <c r="B22" s="42" t="s">
-        <v>1866</v>
+        <v>1862</v>
       </c>
       <c r="C22" s="42" t="s">
-        <v>1867</v>
+        <v>1863</v>
       </c>
       <c r="D22" s="42" t="s">
-        <v>1868</v>
+        <v>1864</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="4" t="s">
-        <v>1827</v>
+        <v>1823</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>1827</v>
+        <v>1823</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>1869</v>
+        <v>1865</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>1870</v>
+        <v>1866</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="42" t="s">
-        <v>1867</v>
+        <v>1863</v>
       </c>
       <c r="B24" s="42" t="s">
-        <v>1867</v>
+        <v>1863</v>
       </c>
       <c r="C24" s="42" t="s">
-        <v>1819</v>
+        <v>1815</v>
       </c>
       <c r="D24" s="42" t="s">
         <v>1740</v>
@@ -39715,13 +39716,13 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>1871</v>
+        <v>1867</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>1867</v>
+        <v>1863</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>1825</v>
+        <v>1821</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>1734</v>
@@ -39729,13 +39730,13 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="42" t="s">
-        <v>1872</v>
+        <v>1868</v>
       </c>
       <c r="B26" s="42" t="s">
-        <v>1867</v>
+        <v>1863</v>
       </c>
       <c r="C26" s="42" t="s">
-        <v>1826</v>
+        <v>1822</v>
       </c>
       <c r="D26" s="42" t="s">
         <v>1745</v>
@@ -39743,16 +39744,16 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>1873</v>
+        <v>1869</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>1873</v>
+        <v>1869</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>1873</v>
+        <v>1869</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>1874</v>
+        <v>1870</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -39766,18 +39767,18 @@
         <v>510</v>
       </c>
       <c r="D28" s="42" t="s">
-        <v>1875</v>
+        <v>1871</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>1876</v>
+        <v>1872</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>1876</v>
+        <v>1872</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>1825</v>
+        <v>1821</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>1734</v>

</xml_diff>